<commit_message>
ajout des Context sur les extensions pour préciser le champ d'application de l'extension 21b5ae78695a649329f01cb4158624b947a1d3b2
</commit_message>
<xml_diff>
--- a/FL-corrections-structure/ig/StructureDefinition-fr-core-appointment.xlsx
+++ b/FL-corrections-structure/ig/StructureDefinition-fr-core-appointment.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-08T19:18:35+00:00</t>
+    <t>2026-03-11T17:39:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -815,7 +815,7 @@
     <t>The style of appointment or patient that has been booked in the slot (not service type).</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/v2-0276|2.0.0</t>
+    <t>http://terminology.hl7.org/ValueSet/v2-0276|3.0.0</t>
   </si>
   <si>
     <t>.code</t>

</xml_diff>